<commit_message>
Datos BEC actualizados 2026-10-30
</commit_message>
<xml_diff>
--- a/reporte-gas/datos/puntos.xlsx
+++ b/reporte-gas/datos/puntos.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="Raa3d698b5cfe474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="R8807f0972a084330"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,6 +91,56 @@
       </x:c>
       <x:c t="inlineStr">
         <x:is>
+          <x:t>BALLENA</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>Con Interrupciones</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>ND</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>2026 Oct</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>BALLENA</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>Contingencia</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>3258</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>6,21</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>2026 Oct</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
           <x:t>MÁGICO</x:t>
         </x:is>
       </x:c>
@@ -125,11 +175,11 @@
         </x:is>
       </x:c>
       <x:c s="8">
-        <x:v>11648</x:v>
-      </x:c>
-      <x:c t="inlineStr">
-        <x:is>
-          <x:t>19,22</x:t>
+        <x:v>11773</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>19,10</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -166,6 +216,56 @@
       </x:c>
       <x:c t="inlineStr">
         <x:is>
+          <x:t>PLANTA CUPIAGUA</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>Contingencia</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>9117</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>5,68</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>2026 Oct</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>PLANTA CUSIANA</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>Contingencia</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="8">
+        <x:v>14775</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>5,68</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>2026 Oct</x:t>
+        </x:is>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
           <x:t>PLANTA DE GAS DINA</x:t>
         </x:is>
       </x:c>
@@ -5679,7 +5779,7 @@
       </x:c>
       <x:c t="inlineStr">
         <x:is>
-          <x:t>16,66</x:t>
+          <x:t>20,21</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>